<commit_message>
Handling awards with 0 quota
</commit_message>
<xml_diff>
--- a/2025-FLL-Qualifier-Tournaments.xlsx
+++ b/2025-FLL-Qualifier-Tournaments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github-projects\FLL-Season-and-Tournament-Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F28E80CE-93CD-48C4-9332-B20E908E8F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91BD3EC-59B1-40F3-823D-1C4E3D3DC6B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{0852510A-0402-494B-87EA-4B91755641F1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0852510A-0402-494B-87EA-4B91755641F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="9" r:id="rId1"/>
@@ -7776,22 +7776,22 @@
         <v>219</v>
       </c>
       <c r="E15" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F15" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J15" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K15" s="1">
         <v>0</v>
@@ -7806,7 +7806,7 @@
         <v>0</v>
       </c>
       <c r="O15" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>